<commit_message>
end demande scenario reality
</commit_message>
<xml_diff>
--- a/exctraction of data/output/CSV_final_in_excel.xlsx
+++ b/exctraction of data/output/CSV_final_in_excel.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DS33"/>
+  <dimension ref="A1:DT33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -566,6 +566,7 @@
     <col width="20" customWidth="1" min="121" max="121"/>
     <col width="20" customWidth="1" min="122" max="122"/>
     <col width="20" customWidth="1" min="123" max="123"/>
+    <col width="20" customWidth="1" min="124" max="124"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -734,12 +735,13 @@
       <c r="DO1" s="1" t="n"/>
       <c r="DP1" s="1" t="n"/>
       <c r="DQ1" s="1" t="n"/>
-      <c r="DR1" s="1" t="inlineStr">
+      <c r="DR1" s="1" t="n"/>
+      <c r="DS1" s="1" t="inlineStr">
         <is>
           <t>NÚMERO DE VIVIENDAS</t>
         </is>
       </c>
-      <c r="DS1" s="1" t="n"/>
+      <c r="DT1" s="1" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="1" t="n"/>
@@ -927,12 +929,13 @@
       <c r="DO2" s="1" t="n"/>
       <c r="DP2" s="1" t="n"/>
       <c r="DQ2" s="1" t="n"/>
-      <c r="DR2" s="1" t="inlineStr">
+      <c r="DR2" s="1" t="n"/>
+      <c r="DS2" s="1" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="DS2" s="1" t="n"/>
+      <c r="DT2" s="1" t="n"/>
     </row>
     <row r="3" ht="38" customHeight="1">
       <c r="A3" s="1" t="n"/>
@@ -1366,26 +1369,27 @@
         </is>
       </c>
       <c r="DK3" s="1" t="n"/>
-      <c r="DL3" s="1" t="inlineStr">
+      <c r="DL3" s="1" t="n"/>
+      <c r="DM3" s="1" t="inlineStr">
         <is>
           <t>Teléfono</t>
         </is>
       </c>
-      <c r="DM3" s="1" t="n"/>
       <c r="DN3" s="1" t="n"/>
-      <c r="DO3" s="1" t="inlineStr">
+      <c r="DO3" s="1" t="n"/>
+      <c r="DP3" s="1" t="inlineStr">
         <is>
           <t>Internet fijo en la vivienda</t>
         </is>
       </c>
-      <c r="DP3" s="1" t="n"/>
       <c r="DQ3" s="1" t="n"/>
-      <c r="DR3" s="1" t="inlineStr">
+      <c r="DR3" s="1" t="n"/>
+      <c r="DS3" s="1" t="inlineStr">
         <is>
           <t>Hotel, hostal, residencial, alojamiento</t>
         </is>
       </c>
-      <c r="DS3" s="1" t="inlineStr">
+      <c r="DT3" s="1" t="inlineStr">
         <is>
           <t>Hospital o clínica con internación</t>
         </is>
@@ -1711,46 +1715,51 @@
       </c>
       <c r="DJ4" s="1" t="inlineStr">
         <is>
+          <t>Tiene</t>
+        </is>
+      </c>
+      <c r="DK4" s="1" t="inlineStr">
+        <is>
           <t>No tiene</t>
         </is>
       </c>
-      <c r="DK4" s="1" t="inlineStr">
+      <c r="DL4" s="1" t="inlineStr">
         <is>
           <t>Sin especificar</t>
         </is>
       </c>
-      <c r="DL4" s="1" t="inlineStr">
+      <c r="DM4" s="1" t="inlineStr">
         <is>
           <t>Tiene</t>
         </is>
       </c>
-      <c r="DM4" s="1" t="inlineStr">
+      <c r="DN4" s="1" t="inlineStr">
         <is>
           <t>No tiene</t>
         </is>
       </c>
-      <c r="DN4" s="1" t="inlineStr">
+      <c r="DO4" s="1" t="inlineStr">
         <is>
           <t>Sin especificar</t>
         </is>
       </c>
-      <c r="DO4" s="1" t="inlineStr">
+      <c r="DP4" s="1" t="inlineStr">
         <is>
           <t>Tiene</t>
         </is>
       </c>
-      <c r="DP4" s="1" t="inlineStr">
+      <c r="DQ4" s="1" t="inlineStr">
         <is>
           <t>No tiene</t>
         </is>
       </c>
-      <c r="DQ4" s="1" t="inlineStr">
+      <c r="DR4" s="1" t="inlineStr">
         <is>
           <t>Sin especificar</t>
         </is>
       </c>
-      <c r="DR4" s="1" t="inlineStr"/>
       <c r="DS4" s="1" t="inlineStr"/>
+      <c r="DT4" s="1" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -2091,33 +2100,36 @@
         <v>4995</v>
       </c>
       <c r="DJ5" t="n">
+        <v>18233</v>
+      </c>
+      <c r="DK5" t="n">
+        <v>60955</v>
+      </c>
+      <c r="DL5" t="n">
         <v>5021</v>
       </c>
-      <c r="DK5" t="n">
+      <c r="DM5" t="n">
         <v>67903</v>
       </c>
-      <c r="DL5" t="n">
+      <c r="DN5" t="n">
         <v>11306</v>
       </c>
-      <c r="DM5" t="n">
+      <c r="DO5" t="n">
         <v>5000</v>
       </c>
-      <c r="DN5" t="n">
+      <c r="DP5" t="n">
         <v>26147</v>
       </c>
-      <c r="DO5" t="n">
+      <c r="DQ5" t="n">
         <v>53040</v>
       </c>
-      <c r="DP5" t="n">
+      <c r="DR5" t="n">
         <v>5022</v>
       </c>
-      <c r="DQ5" t="n">
-        <v>50093</v>
-      </c>
-      <c r="DR5" t="n">
+      <c r="DS5" t="n">
         <v>398</v>
       </c>
-      <c r="DS5" t="n">
+      <c r="DT5" t="n">
         <v>49</v>
       </c>
     </row>
@@ -2468,33 +2480,36 @@
         <v>231</v>
       </c>
       <c r="DJ6" t="n">
+        <v>365</v>
+      </c>
+      <c r="DK6" t="n">
+        <v>2708</v>
+      </c>
+      <c r="DL6" t="n">
         <v>233</v>
       </c>
-      <c r="DK6" t="n">
+      <c r="DM6" t="n">
         <v>2382</v>
       </c>
-      <c r="DL6" t="n">
+      <c r="DN6" t="n">
         <v>691</v>
       </c>
-      <c r="DM6" t="n">
+      <c r="DO6" t="n">
         <v>233</v>
       </c>
-      <c r="DN6" t="n">
+      <c r="DP6" t="n">
         <v>170</v>
       </c>
-      <c r="DO6" t="n">
+      <c r="DQ6" t="n">
         <v>2903</v>
       </c>
-      <c r="DP6" t="n">
+      <c r="DR6" t="n">
         <v>233</v>
       </c>
-      <c r="DQ6" t="n">
-        <v>1430</v>
-      </c>
-      <c r="DR6" t="n">
+      <c r="DS6" t="n">
         <v>26</v>
       </c>
-      <c r="DS6" t="n">
+      <c r="DT6" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2843,33 +2858,36 @@
         <v>2576</v>
       </c>
       <c r="DJ7" t="n">
+        <v>8135</v>
+      </c>
+      <c r="DK7" t="n">
+        <v>27601</v>
+      </c>
+      <c r="DL7" t="n">
         <v>2597</v>
       </c>
-      <c r="DK7" t="n">
+      <c r="DM7" t="n">
         <v>30728</v>
       </c>
-      <c r="DL7" t="n">
+      <c r="DN7" t="n">
         <v>5021</v>
       </c>
-      <c r="DM7" t="n">
+      <c r="DO7" t="n">
         <v>2584</v>
       </c>
-      <c r="DN7" t="n">
+      <c r="DP7" t="n">
         <v>13447</v>
       </c>
-      <c r="DO7" t="n">
+      <c r="DQ7" t="n">
         <v>22293</v>
       </c>
-      <c r="DP7" t="n">
+      <c r="DR7" t="n">
         <v>2593</v>
       </c>
-      <c r="DQ7" t="n">
-        <v>22959</v>
-      </c>
-      <c r="DR7" t="n">
+      <c r="DS7" t="n">
         <v>146</v>
       </c>
-      <c r="DS7" t="n">
+      <c r="DT7" t="n">
         <v>16</v>
       </c>
     </row>
@@ -3220,33 +3238,36 @@
         <v>1863</v>
       </c>
       <c r="DJ8" t="n">
+        <v>5833</v>
+      </c>
+      <c r="DK8" t="n">
+        <v>19729</v>
+      </c>
+      <c r="DL8" t="n">
         <v>1880</v>
       </c>
-      <c r="DK8" t="n">
+      <c r="DM8" t="n">
         <v>22190</v>
       </c>
-      <c r="DL8" t="n">
+      <c r="DN8" t="n">
         <v>3383</v>
       </c>
-      <c r="DM8" t="n">
+      <c r="DO8" t="n">
         <v>1869</v>
       </c>
-      <c r="DN8" t="n">
+      <c r="DP8" t="n">
         <v>9476</v>
       </c>
-      <c r="DO8" t="n">
+      <c r="DQ8" t="n">
         <v>16090</v>
       </c>
-      <c r="DP8" t="n">
+      <c r="DR8" t="n">
         <v>1876</v>
       </c>
-      <c r="DQ8" t="n">
-        <v>16724</v>
-      </c>
-      <c r="DR8" t="n">
+      <c r="DS8" t="n">
         <v>40</v>
       </c>
-      <c r="DS8" t="n">
+      <c r="DT8" t="n">
         <v>8</v>
       </c>
     </row>
@@ -3597,33 +3618,36 @@
         <v>713</v>
       </c>
       <c r="DJ9" t="n">
+        <v>2302</v>
+      </c>
+      <c r="DK9" t="n">
+        <v>7872</v>
+      </c>
+      <c r="DL9" t="n">
         <v>717</v>
       </c>
-      <c r="DK9" t="n">
+      <c r="DM9" t="n">
         <v>8538</v>
       </c>
-      <c r="DL9" t="n">
+      <c r="DN9" t="n">
         <v>1638</v>
       </c>
-      <c r="DM9" t="n">
+      <c r="DO9" t="n">
         <v>715</v>
       </c>
-      <c r="DN9" t="n">
+      <c r="DP9" t="n">
         <v>3971</v>
       </c>
-      <c r="DO9" t="n">
+      <c r="DQ9" t="n">
         <v>6203</v>
       </c>
-      <c r="DP9" t="n">
+      <c r="DR9" t="n">
         <v>717</v>
       </c>
-      <c r="DQ9" t="n">
-        <v>6235</v>
-      </c>
-      <c r="DR9" t="n">
+      <c r="DS9" t="n">
         <v>106</v>
       </c>
-      <c r="DS9" t="n">
+      <c r="DT9" t="n">
         <v>8</v>
       </c>
     </row>
@@ -3974,33 +3998,36 @@
         <v>173</v>
       </c>
       <c r="DJ10" t="n">
+        <v>477</v>
+      </c>
+      <c r="DK10" t="n">
+        <v>2766</v>
+      </c>
+      <c r="DL10" t="n">
         <v>174</v>
       </c>
-      <c r="DK10" t="n">
+      <c r="DM10" t="n">
         <v>2718</v>
       </c>
-      <c r="DL10" t="n">
+      <c r="DN10" t="n">
         <v>525</v>
       </c>
-      <c r="DM10" t="n">
+      <c r="DO10" t="n">
         <v>174</v>
       </c>
-      <c r="DN10" t="n">
+      <c r="DP10" t="n">
         <v>726</v>
       </c>
-      <c r="DO10" t="n">
+      <c r="DQ10" t="n">
         <v>2517</v>
       </c>
-      <c r="DP10" t="n">
+      <c r="DR10" t="n">
         <v>174</v>
       </c>
-      <c r="DQ10" t="n">
-        <v>1955</v>
-      </c>
-      <c r="DR10" t="n">
+      <c r="DS10" t="n">
         <v>7</v>
       </c>
-      <c r="DS10" t="n">
+      <c r="DT10" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4351,33 +4378,36 @@
         <v>168</v>
       </c>
       <c r="DJ11" t="n">
+        <v>383</v>
+      </c>
+      <c r="DK11" t="n">
+        <v>2202</v>
+      </c>
+      <c r="DL11" t="n">
         <v>170</v>
       </c>
-      <c r="DK11" t="n">
+      <c r="DM11" t="n">
         <v>2264</v>
       </c>
-      <c r="DL11" t="n">
+      <c r="DN11" t="n">
         <v>321</v>
       </c>
-      <c r="DM11" t="n">
+      <c r="DO11" t="n">
         <v>170</v>
       </c>
-      <c r="DN11" t="n">
+      <c r="DP11" t="n">
         <v>635</v>
       </c>
-      <c r="DO11" t="n">
+      <c r="DQ11" t="n">
         <v>1949</v>
       </c>
-      <c r="DP11" t="n">
+      <c r="DR11" t="n">
         <v>171</v>
       </c>
-      <c r="DQ11" t="n">
-        <v>1724</v>
-      </c>
-      <c r="DR11" t="n">
+      <c r="DS11" t="n">
         <v>18</v>
       </c>
-      <c r="DS11" t="n">
+      <c r="DT11" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4728,33 +4758,36 @@
         <v>120</v>
       </c>
       <c r="DJ12" t="n">
+        <v>93</v>
+      </c>
+      <c r="DK12" t="n">
+        <v>1242</v>
+      </c>
+      <c r="DL12" t="n">
         <v>120</v>
       </c>
-      <c r="DK12" t="n">
+      <c r="DM12" t="n">
         <v>1004</v>
       </c>
-      <c r="DL12" t="n">
+      <c r="DN12" t="n">
         <v>332</v>
       </c>
-      <c r="DM12" t="n">
+      <c r="DO12" t="n">
         <v>119</v>
       </c>
-      <c r="DN12" t="n">
+      <c r="DP12" t="n">
         <v>58</v>
       </c>
-      <c r="DO12" t="n">
+      <c r="DQ12" t="n">
         <v>1277</v>
       </c>
-      <c r="DP12" t="n">
+      <c r="DR12" t="n">
         <v>120</v>
       </c>
-      <c r="DQ12" t="n">
-        <v>557</v>
-      </c>
-      <c r="DR12" t="n">
+      <c r="DS12" t="n">
         <v>7</v>
       </c>
-      <c r="DS12" t="n">
+      <c r="DT12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5101,33 +5134,36 @@
         <v>1727</v>
       </c>
       <c r="DJ13" t="n">
+        <v>8780</v>
+      </c>
+      <c r="DK13" t="n">
+        <v>24436</v>
+      </c>
+      <c r="DL13" t="n">
         <v>1727</v>
       </c>
-      <c r="DK13" t="n">
+      <c r="DM13" t="n">
         <v>28807</v>
       </c>
-      <c r="DL13" t="n">
+      <c r="DN13" t="n">
         <v>4416</v>
       </c>
-      <c r="DM13" t="n">
+      <c r="DO13" t="n">
         <v>1720</v>
       </c>
-      <c r="DN13" t="n">
+      <c r="DP13" t="n">
         <v>11111</v>
       </c>
-      <c r="DO13" t="n">
+      <c r="DQ13" t="n">
         <v>22101</v>
       </c>
-      <c r="DP13" t="n">
+      <c r="DR13" t="n">
         <v>1731</v>
       </c>
-      <c r="DQ13" t="n">
-        <v>21468</v>
-      </c>
-      <c r="DR13" t="n">
+      <c r="DS13" t="n">
         <v>194</v>
       </c>
-      <c r="DS13" t="n">
+      <c r="DT13" t="n">
         <v>27</v>
       </c>
     </row>
@@ -5476,33 +5512,36 @@
         <v>815</v>
       </c>
       <c r="DJ14" t="n">
+        <v>7071</v>
+      </c>
+      <c r="DK14" t="n">
+        <v>11944</v>
+      </c>
+      <c r="DL14" t="n">
         <v>816</v>
       </c>
-      <c r="DK14" t="n">
+      <c r="DM14" t="n">
         <v>17415</v>
       </c>
-      <c r="DL14" t="n">
+      <c r="DN14" t="n">
         <v>1600</v>
       </c>
-      <c r="DM14" t="n">
+      <c r="DO14" t="n">
         <v>816</v>
       </c>
-      <c r="DN14" t="n">
+      <c r="DP14" t="n">
         <v>10110</v>
       </c>
-      <c r="DO14" t="n">
+      <c r="DQ14" t="n">
         <v>8904</v>
       </c>
-      <c r="DP14" t="n">
+      <c r="DR14" t="n">
         <v>817</v>
       </c>
-      <c r="DQ14" t="n">
-        <v>13598</v>
-      </c>
-      <c r="DR14" t="n">
+      <c r="DS14" t="n">
         <v>112</v>
       </c>
-      <c r="DS14" t="n">
+      <c r="DT14" t="n">
         <v>14</v>
       </c>
     </row>
@@ -5853,33 +5892,36 @@
         <v>545</v>
       </c>
       <c r="DJ15" t="n">
+        <v>6473</v>
+      </c>
+      <c r="DK15" t="n">
+        <v>8545</v>
+      </c>
+      <c r="DL15" t="n">
         <v>546</v>
       </c>
-      <c r="DK15" t="n">
+      <c r="DM15" t="n">
         <v>14080</v>
       </c>
-      <c r="DL15" t="n">
+      <c r="DN15" t="n">
         <v>938</v>
       </c>
-      <c r="DM15" t="n">
+      <c r="DO15" t="n">
         <v>546</v>
       </c>
-      <c r="DN15" t="n">
+      <c r="DP15" t="n">
         <v>9430</v>
       </c>
-      <c r="DO15" t="n">
+      <c r="DQ15" t="n">
         <v>5587</v>
       </c>
-      <c r="DP15" t="n">
+      <c r="DR15" t="n">
         <v>547</v>
       </c>
-      <c r="DQ15" t="n">
-        <v>11192</v>
-      </c>
-      <c r="DR15" t="n">
+      <c r="DS15" t="n">
         <v>102</v>
       </c>
-      <c r="DS15" t="n">
+      <c r="DT15" t="n">
         <v>8</v>
       </c>
     </row>
@@ -6230,33 +6272,36 @@
         <v>177</v>
       </c>
       <c r="DJ16" t="n">
+        <v>405</v>
+      </c>
+      <c r="DK16" t="n">
+        <v>1648</v>
+      </c>
+      <c r="DL16" t="n">
         <v>177</v>
       </c>
-      <c r="DK16" t="n">
+      <c r="DM16" t="n">
         <v>1716</v>
       </c>
-      <c r="DL16" t="n">
+      <c r="DN16" t="n">
         <v>336</v>
       </c>
-      <c r="DM16" t="n">
+      <c r="DO16" t="n">
         <v>178</v>
       </c>
-      <c r="DN16" t="n">
+      <c r="DP16" t="n">
         <v>547</v>
       </c>
-      <c r="DO16" t="n">
+      <c r="DQ16" t="n">
         <v>1506</v>
       </c>
-      <c r="DP16" t="n">
+      <c r="DR16" t="n">
         <v>177</v>
       </c>
-      <c r="DQ16" t="n">
-        <v>1255</v>
-      </c>
-      <c r="DR16" t="n">
+      <c r="DS16" t="n">
         <v>6</v>
       </c>
-      <c r="DS16" t="n">
+      <c r="DT16" t="n">
         <v>2</v>
       </c>
     </row>
@@ -6607,33 +6652,36 @@
         <v>38</v>
       </c>
       <c r="DJ17" t="n">
+        <v>51</v>
+      </c>
+      <c r="DK17" t="n">
+        <v>713</v>
+      </c>
+      <c r="DL17" t="n">
         <v>38</v>
       </c>
-      <c r="DK17" t="n">
+      <c r="DM17" t="n">
         <v>643</v>
       </c>
-      <c r="DL17" t="n">
+      <c r="DN17" t="n">
         <v>121</v>
       </c>
-      <c r="DM17" t="n">
+      <c r="DO17" t="n">
         <v>38</v>
       </c>
-      <c r="DN17" t="n">
+      <c r="DP17" t="n">
         <v>15</v>
       </c>
-      <c r="DO17" t="n">
+      <c r="DQ17" t="n">
         <v>749</v>
       </c>
-      <c r="DP17" t="n">
+      <c r="DR17" t="n">
         <v>38</v>
       </c>
-      <c r="DQ17" t="n">
-        <v>512</v>
-      </c>
-      <c r="DR17" t="n">
-        <v>0</v>
-      </c>
       <c r="DS17" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT17" t="n">
         <v>3</v>
       </c>
     </row>
@@ -6984,33 +7032,36 @@
         <v>55</v>
       </c>
       <c r="DJ18" t="n">
+        <v>142</v>
+      </c>
+      <c r="DK18" t="n">
+        <v>1038</v>
+      </c>
+      <c r="DL18" t="n">
         <v>55</v>
       </c>
-      <c r="DK18" t="n">
+      <c r="DM18" t="n">
         <v>976</v>
       </c>
-      <c r="DL18" t="n">
+      <c r="DN18" t="n">
         <v>205</v>
       </c>
-      <c r="DM18" t="n">
+      <c r="DO18" t="n">
         <v>54</v>
       </c>
-      <c r="DN18" t="n">
+      <c r="DP18" t="n">
         <v>118</v>
       </c>
-      <c r="DO18" t="n">
+      <c r="DQ18" t="n">
         <v>1062</v>
       </c>
-      <c r="DP18" t="n">
+      <c r="DR18" t="n">
         <v>55</v>
       </c>
-      <c r="DQ18" t="n">
-        <v>639</v>
-      </c>
-      <c r="DR18" t="n">
+      <c r="DS18" t="n">
         <v>4</v>
       </c>
-      <c r="DS18" t="n">
+      <c r="DT18" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7359,33 +7410,36 @@
         <v>238</v>
       </c>
       <c r="DJ19" t="n">
+        <v>782</v>
+      </c>
+      <c r="DK19" t="n">
+        <v>4095</v>
+      </c>
+      <c r="DL19" t="n">
         <v>238</v>
       </c>
-      <c r="DK19" t="n">
+      <c r="DM19" t="n">
         <v>4061</v>
       </c>
-      <c r="DL19" t="n">
+      <c r="DN19" t="n">
         <v>819</v>
       </c>
-      <c r="DM19" t="n">
+      <c r="DO19" t="n">
         <v>235</v>
       </c>
-      <c r="DN19" t="n">
+      <c r="DP19" t="n">
         <v>425</v>
       </c>
-      <c r="DO19" t="n">
+      <c r="DQ19" t="n">
         <v>4451</v>
       </c>
-      <c r="DP19" t="n">
+      <c r="DR19" t="n">
         <v>239</v>
       </c>
-      <c r="DQ19" t="n">
-        <v>2972</v>
-      </c>
-      <c r="DR19" t="n">
+      <c r="DS19" t="n">
         <v>29</v>
       </c>
-      <c r="DS19" t="n">
+      <c r="DT19" t="n">
         <v>2</v>
       </c>
     </row>
@@ -7736,33 +7790,36 @@
         <v>90</v>
       </c>
       <c r="DJ20" t="n">
+        <v>518</v>
+      </c>
+      <c r="DK20" t="n">
+        <v>1382</v>
+      </c>
+      <c r="DL20" t="n">
         <v>89</v>
       </c>
-      <c r="DK20" t="n">
+      <c r="DM20" t="n">
         <v>1651</v>
       </c>
-      <c r="DL20" t="n">
+      <c r="DN20" t="n">
         <v>251</v>
       </c>
-      <c r="DM20" t="n">
+      <c r="DO20" t="n">
         <v>87</v>
       </c>
-      <c r="DN20" t="n">
+      <c r="DP20" t="n">
         <v>332</v>
       </c>
-      <c r="DO20" t="n">
+      <c r="DQ20" t="n">
         <v>1567</v>
       </c>
-      <c r="DP20" t="n">
+      <c r="DR20" t="n">
         <v>90</v>
       </c>
-      <c r="DQ20" t="n">
-        <v>1307</v>
-      </c>
-      <c r="DR20" t="n">
+      <c r="DS20" t="n">
         <v>26</v>
       </c>
-      <c r="DS20" t="n">
+      <c r="DT20" t="n">
         <v>2</v>
       </c>
     </row>
@@ -8113,33 +8170,36 @@
         <v>48</v>
       </c>
       <c r="DJ21" t="n">
+        <v>27</v>
+      </c>
+      <c r="DK21" t="n">
+        <v>536</v>
+      </c>
+      <c r="DL21" t="n">
         <v>49</v>
       </c>
-      <c r="DK21" t="n">
+      <c r="DM21" t="n">
         <v>364</v>
       </c>
-      <c r="DL21" t="n">
+      <c r="DN21" t="n">
         <v>200</v>
       </c>
-      <c r="DM21" t="n">
+      <c r="DO21" t="n">
         <v>48</v>
       </c>
-      <c r="DN21" t="n">
+      <c r="DP21" t="n">
         <v>2</v>
       </c>
-      <c r="DO21" t="n">
+      <c r="DQ21" t="n">
         <v>561</v>
       </c>
-      <c r="DP21" t="n">
+      <c r="DR21" t="n">
         <v>49</v>
       </c>
-      <c r="DQ21" t="n">
-        <v>220</v>
-      </c>
-      <c r="DR21" t="n">
+      <c r="DS21" t="n">
         <v>1</v>
       </c>
-      <c r="DS21" t="n">
+      <c r="DT21" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8490,33 +8550,36 @@
         <v>100</v>
       </c>
       <c r="DJ22" t="n">
+        <v>237</v>
+      </c>
+      <c r="DK22" t="n">
+        <v>2177</v>
+      </c>
+      <c r="DL22" t="n">
         <v>100</v>
       </c>
-      <c r="DK22" t="n">
+      <c r="DM22" t="n">
         <v>2046</v>
       </c>
-      <c r="DL22" t="n">
+      <c r="DN22" t="n">
         <v>368</v>
       </c>
-      <c r="DM22" t="n">
+      <c r="DO22" t="n">
         <v>100</v>
       </c>
-      <c r="DN22" t="n">
+      <c r="DP22" t="n">
         <v>91</v>
       </c>
-      <c r="DO22" t="n">
+      <c r="DQ22" t="n">
         <v>2323</v>
       </c>
-      <c r="DP22" t="n">
+      <c r="DR22" t="n">
         <v>100</v>
       </c>
-      <c r="DQ22" t="n">
-        <v>1445</v>
-      </c>
-      <c r="DR22" t="n">
+      <c r="DS22" t="n">
         <v>2</v>
       </c>
-      <c r="DS22" t="n">
+      <c r="DT22" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8865,33 +8928,36 @@
         <v>425</v>
       </c>
       <c r="DJ23" t="n">
+        <v>653</v>
+      </c>
+      <c r="DK23" t="n">
+        <v>5613</v>
+      </c>
+      <c r="DL23" t="n">
         <v>424</v>
       </c>
-      <c r="DK23" t="n">
+      <c r="DM23" t="n">
         <v>4935</v>
       </c>
-      <c r="DL23" t="n">
+      <c r="DN23" t="n">
         <v>1331</v>
       </c>
-      <c r="DM23" t="n">
+      <c r="DO23" t="n">
         <v>424</v>
       </c>
-      <c r="DN23" t="n">
+      <c r="DP23" t="n">
         <v>477</v>
       </c>
-      <c r="DO23" t="n">
+      <c r="DQ23" t="n">
         <v>5788</v>
       </c>
-      <c r="DP23" t="n">
+      <c r="DR23" t="n">
         <v>425</v>
       </c>
-      <c r="DQ23" t="n">
-        <v>3351</v>
-      </c>
-      <c r="DR23" t="n">
+      <c r="DS23" t="n">
         <v>49</v>
       </c>
-      <c r="DS23" t="n">
+      <c r="DT23" t="n">
         <v>8</v>
       </c>
     </row>
@@ -9242,33 +9308,36 @@
         <v>150</v>
       </c>
       <c r="DJ24" t="n">
+        <v>193</v>
+      </c>
+      <c r="DK24" t="n">
+        <v>1622</v>
+      </c>
+      <c r="DL24" t="n">
         <v>150</v>
       </c>
-      <c r="DK24" t="n">
+      <c r="DM24" t="n">
         <v>1355</v>
       </c>
-      <c r="DL24" t="n">
+      <c r="DN24" t="n">
         <v>459</v>
       </c>
-      <c r="DM24" t="n">
+      <c r="DO24" t="n">
         <v>151</v>
       </c>
-      <c r="DN24" t="n">
+      <c r="DP24" t="n">
         <v>54</v>
       </c>
-      <c r="DO24" t="n">
+      <c r="DQ24" t="n">
         <v>1760</v>
       </c>
-      <c r="DP24" t="n">
+      <c r="DR24" t="n">
         <v>151</v>
       </c>
-      <c r="DQ24" t="n">
-        <v>970</v>
-      </c>
-      <c r="DR24" t="n">
+      <c r="DS24" t="n">
         <v>9</v>
       </c>
-      <c r="DS24" t="n">
+      <c r="DT24" t="n">
         <v>5</v>
       </c>
     </row>
@@ -9619,33 +9688,36 @@
         <v>113</v>
       </c>
       <c r="DJ25" t="n">
+        <v>176</v>
+      </c>
+      <c r="DK25" t="n">
+        <v>1561</v>
+      </c>
+      <c r="DL25" t="n">
         <v>113</v>
       </c>
-      <c r="DK25" t="n">
+      <c r="DM25" t="n">
         <v>1442</v>
       </c>
-      <c r="DL25" t="n">
+      <c r="DN25" t="n">
         <v>295</v>
       </c>
-      <c r="DM25" t="n">
+      <c r="DO25" t="n">
         <v>113</v>
       </c>
-      <c r="DN25" t="n">
+      <c r="DP25" t="n">
         <v>97</v>
       </c>
-      <c r="DO25" t="n">
+      <c r="DQ25" t="n">
         <v>1640</v>
       </c>
-      <c r="DP25" t="n">
+      <c r="DR25" t="n">
         <v>113</v>
       </c>
-      <c r="DQ25" t="n">
-        <v>983</v>
-      </c>
-      <c r="DR25" t="n">
+      <c r="DS25" t="n">
         <v>9</v>
       </c>
-      <c r="DS25" t="n">
+      <c r="DT25" t="n">
         <v>2</v>
       </c>
     </row>
@@ -9996,33 +10068,36 @@
         <v>162</v>
       </c>
       <c r="DJ26" t="n">
+        <v>284</v>
+      </c>
+      <c r="DK26" t="n">
+        <v>2430</v>
+      </c>
+      <c r="DL26" t="n">
         <v>161</v>
       </c>
-      <c r="DK26" t="n">
+      <c r="DM26" t="n">
         <v>2138</v>
       </c>
-      <c r="DL26" t="n">
+      <c r="DN26" t="n">
         <v>577</v>
       </c>
-      <c r="DM26" t="n">
+      <c r="DO26" t="n">
         <v>160</v>
       </c>
-      <c r="DN26" t="n">
+      <c r="DP26" t="n">
         <v>326</v>
       </c>
-      <c r="DO26" t="n">
+      <c r="DQ26" t="n">
         <v>2388</v>
       </c>
-      <c r="DP26" t="n">
+      <c r="DR26" t="n">
         <v>161</v>
       </c>
-      <c r="DQ26" t="n">
-        <v>1398</v>
-      </c>
-      <c r="DR26" t="n">
+      <c r="DS26" t="n">
         <v>31</v>
       </c>
-      <c r="DS26" t="n">
+      <c r="DT26" t="n">
         <v>1</v>
       </c>
     </row>
@@ -10371,33 +10446,36 @@
         <v>83</v>
       </c>
       <c r="DJ27" t="n">
+        <v>164</v>
+      </c>
+      <c r="DK27" t="n">
+        <v>1262</v>
+      </c>
+      <c r="DL27" t="n">
         <v>83</v>
       </c>
-      <c r="DK27" t="n">
+      <c r="DM27" t="n">
         <v>1161</v>
       </c>
-      <c r="DL27" t="n">
+      <c r="DN27" t="n">
         <v>265</v>
       </c>
-      <c r="DM27" t="n">
+      <c r="DO27" t="n">
         <v>83</v>
       </c>
-      <c r="DN27" t="n">
+      <c r="DP27" t="n">
         <v>56</v>
       </c>
-      <c r="DO27" t="n">
+      <c r="DQ27" t="n">
         <v>1369</v>
       </c>
-      <c r="DP27" t="n">
+      <c r="DR27" t="n">
         <v>84</v>
       </c>
-      <c r="DQ27" t="n">
-        <v>748</v>
-      </c>
-      <c r="DR27" t="n">
+      <c r="DS27" t="n">
         <v>2</v>
       </c>
-      <c r="DS27" t="n">
+      <c r="DT27" t="n">
         <v>1</v>
       </c>
     </row>
@@ -10748,33 +10826,36 @@
         <v>45</v>
       </c>
       <c r="DJ28" t="n">
+        <v>121</v>
+      </c>
+      <c r="DK28" t="n">
+        <v>695</v>
+      </c>
+      <c r="DL28" t="n">
         <v>44</v>
       </c>
-      <c r="DK28" t="n">
+      <c r="DM28" t="n">
         <v>681</v>
       </c>
-      <c r="DL28" t="n">
+      <c r="DN28" t="n">
         <v>134</v>
       </c>
-      <c r="DM28" t="n">
+      <c r="DO28" t="n">
         <v>45</v>
       </c>
-      <c r="DN28" t="n">
+      <c r="DP28" t="n">
         <v>35</v>
       </c>
-      <c r="DO28" t="n">
+      <c r="DQ28" t="n">
         <v>780</v>
       </c>
-      <c r="DP28" t="n">
+      <c r="DR28" t="n">
         <v>45</v>
       </c>
-      <c r="DQ28" t="n">
-        <v>518</v>
-      </c>
-      <c r="DR28" t="n">
+      <c r="DS28" t="n">
         <v>1</v>
       </c>
-      <c r="DS28" t="n">
+      <c r="DT28" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11125,33 +11206,36 @@
         <v>38</v>
       </c>
       <c r="DJ29" t="n">
+        <v>43</v>
+      </c>
+      <c r="DK29" t="n">
+        <v>567</v>
+      </c>
+      <c r="DL29" t="n">
         <v>39</v>
       </c>
-      <c r="DK29" t="n">
+      <c r="DM29" t="n">
         <v>480</v>
       </c>
-      <c r="DL29" t="n">
+      <c r="DN29" t="n">
         <v>131</v>
       </c>
-      <c r="DM29" t="n">
+      <c r="DO29" t="n">
         <v>38</v>
       </c>
-      <c r="DN29" t="n">
+      <c r="DP29" t="n">
         <v>21</v>
       </c>
-      <c r="DO29" t="n">
+      <c r="DQ29" t="n">
         <v>589</v>
       </c>
-      <c r="DP29" t="n">
+      <c r="DR29" t="n">
         <v>39</v>
       </c>
-      <c r="DQ29" t="n">
-        <v>230</v>
-      </c>
-      <c r="DR29" t="n">
+      <c r="DS29" t="n">
         <v>1</v>
       </c>
-      <c r="DS29" t="n">
+      <c r="DT29" t="n">
         <v>1</v>
       </c>
     </row>
@@ -11500,33 +11584,36 @@
         <v>166</v>
       </c>
       <c r="DJ30" t="n">
+        <v>110</v>
+      </c>
+      <c r="DK30" t="n">
+        <v>1522</v>
+      </c>
+      <c r="DL30" t="n">
         <v>166</v>
       </c>
-      <c r="DK30" t="n">
+      <c r="DM30" t="n">
         <v>1235</v>
       </c>
-      <c r="DL30" t="n">
+      <c r="DN30" t="n">
         <v>401</v>
       </c>
-      <c r="DM30" t="n">
+      <c r="DO30" t="n">
         <v>162</v>
       </c>
-      <c r="DN30" t="n">
+      <c r="DP30" t="n">
         <v>43</v>
       </c>
-      <c r="DO30" t="n">
+      <c r="DQ30" t="n">
         <v>1589</v>
       </c>
-      <c r="DP30" t="n">
+      <c r="DR30" t="n">
         <v>166</v>
       </c>
-      <c r="DQ30" t="n">
-        <v>799</v>
-      </c>
-      <c r="DR30" t="n">
+      <c r="DS30" t="n">
         <v>2</v>
       </c>
-      <c r="DS30" t="n">
+      <c r="DT30" t="n">
         <v>2</v>
       </c>
     </row>
@@ -11877,33 +11964,36 @@
         <v>21</v>
       </c>
       <c r="DJ31" t="n">
+        <v>49</v>
+      </c>
+      <c r="DK31" t="n">
+        <v>419</v>
+      </c>
+      <c r="DL31" t="n">
         <v>21</v>
       </c>
-      <c r="DK31" t="n">
+      <c r="DM31" t="n">
         <v>367</v>
       </c>
-      <c r="DL31" t="n">
+      <c r="DN31" t="n">
         <v>101</v>
       </c>
-      <c r="DM31" t="n">
+      <c r="DO31" t="n">
         <v>21</v>
       </c>
-      <c r="DN31" t="n">
+      <c r="DP31" t="n">
         <v>19</v>
       </c>
-      <c r="DO31" t="n">
+      <c r="DQ31" t="n">
         <v>449</v>
       </c>
-      <c r="DP31" t="n">
+      <c r="DR31" t="n">
         <v>21</v>
       </c>
-      <c r="DQ31" t="n">
-        <v>261</v>
-      </c>
-      <c r="DR31" t="n">
+      <c r="DS31" t="n">
         <v>1</v>
       </c>
-      <c r="DS31" t="n">
+      <c r="DT31" t="n">
         <v>1</v>
       </c>
     </row>
@@ -12254,33 +12344,36 @@
         <v>78</v>
       </c>
       <c r="DJ32" t="n">
+        <v>35</v>
+      </c>
+      <c r="DK32" t="n">
+        <v>595</v>
+      </c>
+      <c r="DL32" t="n">
         <v>78</v>
       </c>
-      <c r="DK32" t="n">
+      <c r="DM32" t="n">
         <v>471</v>
       </c>
-      <c r="DL32" t="n">
+      <c r="DN32" t="n">
         <v>163</v>
       </c>
-      <c r="DM32" t="n">
+      <c r="DO32" t="n">
         <v>74</v>
       </c>
-      <c r="DN32" t="n">
+      <c r="DP32" t="n">
         <v>16</v>
       </c>
-      <c r="DO32" t="n">
+      <c r="DQ32" t="n">
         <v>614</v>
       </c>
-      <c r="DP32" t="n">
+      <c r="DR32" t="n">
         <v>78</v>
       </c>
-      <c r="DQ32" t="n">
-        <v>324</v>
-      </c>
-      <c r="DR32" t="n">
+      <c r="DS32" t="n">
         <v>1</v>
       </c>
-      <c r="DS32" t="n">
+      <c r="DT32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12631,33 +12724,36 @@
         <v>67</v>
       </c>
       <c r="DJ33" t="n">
+        <v>26</v>
+      </c>
+      <c r="DK33" t="n">
+        <v>508</v>
+      </c>
+      <c r="DL33" t="n">
         <v>67</v>
       </c>
-      <c r="DK33" t="n">
+      <c r="DM33" t="n">
         <v>397</v>
       </c>
-      <c r="DL33" t="n">
+      <c r="DN33" t="n">
         <v>137</v>
       </c>
-      <c r="DM33" t="n">
+      <c r="DO33" t="n">
         <v>67</v>
       </c>
-      <c r="DN33" t="n">
+      <c r="DP33" t="n">
         <v>8</v>
       </c>
-      <c r="DO33" t="n">
+      <c r="DQ33" t="n">
         <v>526</v>
       </c>
-      <c r="DP33" t="n">
+      <c r="DR33" t="n">
         <v>67</v>
       </c>
-      <c r="DQ33" t="n">
-        <v>214</v>
-      </c>
-      <c r="DR33" t="n">
-        <v>0</v>
-      </c>
       <c r="DS33" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT33" t="n">
         <v>1</v>
       </c>
     </row>
@@ -12667,9 +12763,11 @@
     <mergeCell ref="BE3:BF3"/>
     <mergeCell ref="CE3:CG3"/>
     <mergeCell ref="BG3:BH3"/>
-    <mergeCell ref="CK1:DQ1"/>
+    <mergeCell ref="DS1:DT1"/>
     <mergeCell ref="BR3:BT3"/>
     <mergeCell ref="CB3:CD3"/>
+    <mergeCell ref="DJ3:DL3"/>
+    <mergeCell ref="DP3:DR3"/>
     <mergeCell ref="CY3:CZ3"/>
     <mergeCell ref="DA3:DB3"/>
     <mergeCell ref="CL3:CM3"/>
@@ -12682,37 +12780,35 @@
     <mergeCell ref="BN2:BT2"/>
     <mergeCell ref="BD2:BH2"/>
     <mergeCell ref="CS3:CT3"/>
-    <mergeCell ref="DJ3:DK3"/>
     <mergeCell ref="CR2:DB2"/>
     <mergeCell ref="B1:B4"/>
     <mergeCell ref="AD1:BC1"/>
     <mergeCell ref="O2:T2"/>
     <mergeCell ref="AA2:AC2"/>
-    <mergeCell ref="DL3:DN3"/>
     <mergeCell ref="BV3:BX3"/>
     <mergeCell ref="U1:AC1"/>
     <mergeCell ref="BU2:CJ2"/>
     <mergeCell ref="DG3:DI3"/>
     <mergeCell ref="CN3:CO3"/>
     <mergeCell ref="AD2:AK2"/>
+    <mergeCell ref="DC2:DR2"/>
     <mergeCell ref="CP3:CQ3"/>
     <mergeCell ref="AU2:BC2"/>
     <mergeCell ref="F1:T1"/>
-    <mergeCell ref="DR2:DS2"/>
+    <mergeCell ref="CK1:DR1"/>
+    <mergeCell ref="DS2:DT2"/>
     <mergeCell ref="BD1:BT1"/>
-    <mergeCell ref="DR1:DS1"/>
     <mergeCell ref="X2:Z2"/>
     <mergeCell ref="CH3:CJ3"/>
     <mergeCell ref="BJ3:BK3"/>
     <mergeCell ref="CK2:CQ2"/>
     <mergeCell ref="BL3:BM3"/>
     <mergeCell ref="I2:N2"/>
-    <mergeCell ref="DO3:DQ3"/>
+    <mergeCell ref="DM3:DO3"/>
     <mergeCell ref="DD3:DF3"/>
     <mergeCell ref="AL2:AT2"/>
     <mergeCell ref="BU1:CJ1"/>
     <mergeCell ref="CU3:CV3"/>
-    <mergeCell ref="DC2:DQ2"/>
     <mergeCell ref="CW3:CX3"/>
     <mergeCell ref="D1:D4"/>
     <mergeCell ref="BY3:CA3"/>

</xml_diff>